<commit_message>
schema do banco com FK/PK completas; atualiza de-para com achados de CNPJ/CNES e tratamento de nulos
</commit_message>
<xml_diff>
--- a/docs/de-para/de_para_p5_capacidade_hospitalar.xlsx
+++ b/docs/de-para/de_para_p5_capacidade_hospitalar.xlsx
@@ -1049,7 +1049,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>Perguntas 2, 3, 4, 5, 6 — ATENÇÃO: liga com as outras tabelas por CNPJ (cgc_hosp), não por CNES; precisa de tradução</t>
+          <t>Perguntas 2, 3, 4, 5, 6 — liga com CNES-LT via de_para_cnpj_cnes (cgc_hosp=cpf_cnpj, resolvido); cgc_hosp pode ser NULL (17.695 casos, jul-dez/2024) — sempre LEFT JOIN</t>
         </is>
       </c>
     </row>
@@ -2320,7 +2320,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>FK (revisado)</t>
+          <t>FK, NULLABLE</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>CORRIGIDO: campo 'CNES' NÃO existe no SIH-RD isolado — o identificador aqui é CNPJ, não código CNES. Precisa de tabela de tradução CNPJ&lt;-&gt;CNES para juntar com fato_leitos e dim_estabelecimento — pendência real de arquitetura.</t>
+          <t>RESOLVIDO (18-20/09): CNPJ do CGC_HOSP bate diretamente com CPF_CNPJ do CNES-LT (39.986/54.297 confirmados em teste real) — não precisa de fonte externa. MAS pode vir vazio (''): converter para NULL no 02_transformacao.py, manter a linha, sempre LEFT JOIN (nunca INNER).</t>
         </is>
       </c>
     </row>
@@ -2743,6 +2743,20 @@
       <c r="A16" s="11" t="inlineStr">
         <is>
           <t>ALERTA 1: 'CNES' havia sido marcado erroneamente como FK antes — o campo real é CGC_HOSP (CNPJ). ALERTA 2: DT_SAIDA e MUNIC_MOV foram CONFIRMADOS com dado real (antes constavam como pendentes) — ambos object/texto. ALERTA 3: todos os campos do RD chegam como 'object' (texto), inclusive DIAS_PERM e IDADE. Conversão obrigatória antes de qualquer cálculo numérico no 02_transformacao.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>ALERTA 4 (20/09, validado com dado real): CGC_HOSP vem VAZIO ('') em 17.695 registros de Recife, competências jul-dez/2024. DECISÃO DE ARQUITETURA CONFIRMADA: converter '' em NULL no 02_transformacao.py; NUNCA descartar a internação; sempre LEFT JOIN (nunca INNER) entre fato_internacoes e dim_estabelecimento/de_para_cnpj_cnes — INNER JOIN perderia ~17.695 internações reais. No painel: COALESCE(nome, 'Hospital não identificado'), nunca célula vazia.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="11" t="inlineStr">
+        <is>
+          <t>ALERTA 5 (PADRÃO A INVESTIGAR): os vazios de CGC_HOSP NÃO seguem o padrão esperado de 'mais recente = mais incompleto'. Contagem por competência (jul-dez/2024): 202407=4606, 202410=4525, 202411=3979, 202412=4585 — mas 202408 e 202409 não aparecem (zero vazios, ou arquivo ausente — a confirmar). Jul/2024 tem quase tanto vazio quanto dez/2024, apesar de ser 1+ ano mais antigo — contradiz a hipótese de que é só defasagem de processamento do SIH. Investigar antes de tratar como resolvido.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
FIX: Padronização da sigla MHSL na documentação e Schema
</commit_message>
<xml_diff>
--- a/docs/de-para/de_para_p5_capacidade_hospitalar.xlsx
+++ b/docs/de-para/de_para_p5_capacidade_hospitalar.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leia-me" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tabelas do Banco" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CNES_LT_Leitos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hospitais_MS_Estab" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MSHL_Estab" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SIH_RD_Internacoes" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dominio_TP_LEITO" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dominio_CODLEITO" sheetId="7" state="visible" r:id="rId7"/>
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -563,7 +563,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Aba 'Hospitais_MS_Estab'    — de-para de campos da fonte de estabelecimentos (Hospitais e Leitos/Ministério da Saúde).</t>
+          <t>Aba 'MSHL_Estab'            — de-para de campos da fonte de estabelecimentos (MSHL — Hospitais e Leitos/Ministério da Saúde).</t>
         </is>
       </c>
     </row>
@@ -710,133 +710,140 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>Hospitais e Leitos (MS): fonte agora EXPLICITAMENTE validada pelo Canvas atualizado (citada nas Perguntas 1 e 5 como</t>
+          <t>MSHL (Hospitais e Leitos/MS): sigla adotada pelo time (20/09), mesmo padrão de LT/RD. Fonte agora EXPLICITAMENTE</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         fonte oficial de identificação dos hospitais) — deixou de ser uma escolha provisória da engenharia e passou a</t>
+          <t>validada pelo Canvas atualizado (citada nas Perguntas 1 e 5 como</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         ser parte confirmada do desenho de negócio. Ainda assim, não existe dicionário oficial com PK/FK para esta</t>
+          <t xml:space="preserve">         fonte oficial de identificação dos hospitais) — deixou de ser uma escolha provisória da engenharia e passou a</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         fonte (não é uma tabela do CNES) — a chave primária proposta (CNES + COMP) continua sendo uma INFERÊNCIA</t>
+          <t xml:space="preserve">         ser parte confirmada do desenho de negócio. Ainda assim, não existe dicionário oficial com PK/FK para esta</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">         fonte (não é uma tabela do CNES) — a chave primária proposta (CNES + COMP) continua sendo uma INFERÊNCIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">         baseada no formato dos dados observados, não uma definição documentada pelo Ministério da Saúde.</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr"/>
-    </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>SIH-RD: o caderno de layout oficial do SIH AINDA NÃO foi localizado pelo time (o arquivo baixado do site do CNES,</t>
-        </is>
-      </c>
+      <c r="A39" s="3" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         apesar do nome, continha apenas o layout do CNES). Por isso, esta aba cobre só os campos usados pelas</t>
+          <t>SIH-RD: o caderno de layout oficial do SIH AINDA NÃO foi localizado pelo time (o arquivo baixado do site do CNES,</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         perguntas do Canvas, com descrição reconstruída de fontes públicas (ver docs/dicionario_dominios_sih_rd.md) —</t>
+          <t xml:space="preserve">         apesar do nome, continha apenas o layout do CNES). Por isso, esta aba cobre só os campos usados pelas</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">         SEM confirmação oficial de PK/FK. Tratar como rascunho até a documentação oficial do SIH ser encontrada.</t>
+          <t xml:space="preserve">         perguntas do Canvas, com descrição reconstruída de fontes públicas (ver docs/dicionario_dominios_sih_rd.md) —</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
+          <t xml:space="preserve">         SEM confirmação oficial de PK/FK. Tratar como rascunho até a documentação oficial do SIH ser encontrada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
           <t xml:space="preserve">         DT_SAIDA e MUNIC_MOV foram confirmados existindo no dado real, com dtype object (texto), formato AAAAMMDD.</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="3" t="inlineStr"/>
-    </row>
     <row r="45">
-      <c r="A45" s="3" t="inlineStr">
+      <c r="A45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>ACHADO CRÍTICO SOBRE TIPOS DE DADO (confirmado rodando pandas .dtypes nos arquivos reais)</t>
         </is>
       </c>
     </row>
-    <row r="46">
-      <c r="A46" s="3" t="inlineStr"/>
-    </row>
     <row r="47">
-      <c r="A47" s="3" t="inlineStr">
-        <is>
-          <t>CNES-LT e SIH-RD chegam do PySUS com TODOS os campos como 'object' (texto) — mesmo os numéricos, como QT_EXIST,</t>
-        </is>
-      </c>
+      <c r="A47" s="3" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>QT_SUS, DIAS_PERM e IDADE. Já a fonte Hospitais e Leitos (MS) chega com tipo real (int64/float64/object). Isso tem</t>
+          <t>CNES-LT e SIH-RD chegam do PySUS com TODOS os campos como 'object' (texto) — mesmo os numéricos, como QT_EXIST,</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>duas consequências práticas para o 02_transformacao.py:</t>
+          <t>QT_SUS, DIAS_PERM e IDADE. Já a fonte MSHL chega com tipo real (int64/float64/object). Isso tem</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>1) Campos numéricos de CNES-LT e SIH-RD precisam de conversão explícita (pd.to_numeric) antes de qualquer soma,</t>
+          <t>duas consequências práticas para o 02_transformacao.py:</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   média ou comparação — hoje eles se comportariam como texto (ex.: ordenaria '10' antes de '9').</t>
+          <t>1) Campos numéricos de CNES-LT e SIH-RD precisam de conversão explícita (pd.to_numeric) antes de qualquer soma,</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>2) O campo CNES aparece com tipos diferentes em fontes diferentes (object no CNES-LT/SIH-RD via CGC_HOSP-&gt;CNES,</t>
+          <t xml:space="preserve">   média ou comparação — hoje eles se comportariam como texto (ex.: ordenaria '10' antes de '9').</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>2) O campo CNES aparece com tipos diferentes em fontes diferentes (object no CNES-LT/SIH-RD via CGC_HOSP-&gt;CNES,</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">   int64 na fonte MS) — os tipos precisam ser padronizados antes de qualquer junção (join) entre as tabelas.</t>
         </is>
@@ -997,7 +1004,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Hospitais e Leitos (Ministério da Saúde) — fonte confirmada no Canvas</t>
+          <t>MSHL — Hospitais e Leitos (Ministério da Saúde) — fonte confirmada no Canvas</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">

</xml_diff>